<commit_message>
add computer-generated and morphed federal cases
</commit_message>
<xml_diff>
--- a/Pfefferkorn & Demeocq - AI-CSAM Prosecutions Dataset (2026-09-21).xlsx
+++ b/Pfefferkorn & Demeocq - AI-CSAM Prosecutions Dataset (2026-09-21).xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1377" uniqueCount="482">
   <si>
     <t>Title</t>
   </si>
@@ -1572,6 +1572,36 @@
   <si>
     <t>Outcome 
 (as of 9/21/2026)</t>
+  </si>
+  <si>
+    <t>U.S. v. Holst</t>
+  </si>
+  <si>
+    <t>5:22-cr-50022</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/69248969/united-states-v-holst/</t>
+  </si>
+  <si>
+    <t>U.S. v. Clark</t>
+  </si>
+  <si>
+    <t>2:25-cr-00061</t>
+  </si>
+  <si>
+    <t>E.D. Ky.</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/73437702/united-states-v-clark/</t>
+  </si>
+  <si>
+    <t>U.S. v. Dion</t>
+  </si>
+  <si>
+    <t>1:25-cr-00052</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/69647758/united-states-v-dion/</t>
   </si>
 </sst>
 </file>
@@ -6944,6 +6974,123 @@
       <c r="V72" s="3"/>
       <c r="W72" s="3"/>
     </row>
+    <row r="73" spans="1:23" ht="13" x14ac:dyDescent="0.15">
+      <c r="A73" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="E73" s="5">
+        <v>44609</v>
+      </c>
+      <c r="F73" s="3">
+        <v>2022</v>
+      </c>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3"/>
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+      <c r="K73" s="3"/>
+      <c r="L73" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="M73" s="3"/>
+      <c r="N73" s="3"/>
+      <c r="O73" s="3"/>
+      <c r="P73" s="3"/>
+      <c r="Q73" s="3"/>
+      <c r="R73" s="3"/>
+      <c r="S73" s="3"/>
+      <c r="T73" s="3"/>
+      <c r="U73" s="3"/>
+      <c r="V73" s="3"/>
+      <c r="W73" s="3"/>
+    </row>
+    <row r="74" spans="1:23" ht="13" x14ac:dyDescent="0.15">
+      <c r="A74" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E74" s="5">
+        <v>45883</v>
+      </c>
+      <c r="F74" s="3">
+        <v>2025</v>
+      </c>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
+      <c r="I74" s="3"/>
+      <c r="J74" s="3"/>
+      <c r="K74" s="3"/>
+      <c r="L74" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="M74" s="3"/>
+      <c r="N74" s="3"/>
+      <c r="O74" s="3"/>
+      <c r="P74" s="3"/>
+      <c r="Q74" s="3"/>
+      <c r="R74" s="3"/>
+      <c r="S74" s="3"/>
+      <c r="T74" s="3"/>
+      <c r="U74" s="3"/>
+      <c r="V74" s="3"/>
+      <c r="W74" s="3"/>
+    </row>
+    <row r="75" spans="1:23" ht="13" x14ac:dyDescent="0.15">
+      <c r="A75" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="E75" s="5">
+        <v>45701</v>
+      </c>
+      <c r="F75" s="3">
+        <v>2025</v>
+      </c>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+      <c r="K75" s="3"/>
+      <c r="L75" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3"/>
+      <c r="O75" s="3"/>
+      <c r="P75" s="3"/>
+      <c r="Q75" s="3"/>
+      <c r="R75" s="3"/>
+      <c r="S75" s="3"/>
+      <c r="T75" s="3"/>
+      <c r="U75" s="3"/>
+      <c r="V75" s="3"/>
+      <c r="W75" s="3"/>
+    </row>
     <row r="85" spans="1:12" ht="13" x14ac:dyDescent="0.15">
       <c r="E85" s="5"/>
       <c r="I85" s="7"/>
@@ -10128,6 +10275,9 @@
     <hyperlink ref="L71" r:id="rId86" xr:uid="{46030B60-B2D7-7F42-BDE1-3775DC6E74A6}"/>
     <hyperlink ref="L72" r:id="rId87" xr:uid="{44756F98-98DA-3A4D-8D59-8B0C0AB72BF6}"/>
     <hyperlink ref="R60" r:id="rId88" location="docket" xr:uid="{074A3C58-17B2-A349-8396-2028F34BBAB5}"/>
+    <hyperlink ref="L73" r:id="rId93" xr:uid="{8CD84D31-E888-42C8-BC03-C628BE365A66}"/>
+    <hyperlink ref="L74" r:id="rId94" xr:uid="{D3BA6EC1-D474-456B-A0C8-01074B6E3FF0}"/>
+    <hyperlink ref="L75" r:id="rId95" xr:uid="{95616831-A7BF-4E8D-94AC-5A10327E4F3D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId89"/>

</xml_diff>